<commit_message>
Add executive view: section 0 in the plan, page and tracker
</commit_message>
<xml_diff>
--- a/assets/mft-mvp-tracker.xlsx
+++ b/assets/mft-mvp-tracker.xlsx
@@ -8,22 +8,24 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endpoint details" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake options" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake conditions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success criteria" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive view" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endpoint details" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake options" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake conditions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success criteria" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Endpoint details'!$A$4:$G$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Plan'!$A$3:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Dependencies'!$A$4:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data Lake options'!$A$4:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Data Lake conditions'!$A$3:$F$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Success criteria'!$A$3:$F$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Risks'!$A$3:$E$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Executive view'!$A$4:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Endpoint details'!$A$4:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Plan'!$A$3:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Dependencies'!$A$4:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Data Lake options'!$A$4:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Data Lake conditions'!$A$3:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Success criteria'!$A$3:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Risks'!$A$3:$E$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -134,10 +136,10 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -624,6 +626,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Executive view</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>The whole argument on one screen. Detail sits in the tabs to the right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>What we are doing</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Moving one live feed off its legacy transfer mechanisms onto Boomi MFT, and evidencing the result well enough for a go or no-go decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>On what</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Feed ADR.040, the quarterly Migrant Workers Scan. It is the only feed identified that carries both patterns in a single business flow: NPS to ADR internal, and ADR to ONS external.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Monday 28 September to Friday 9 October 2026. Configuration is two days of that.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>What it costs</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Two days of build effort plus about a week of discovery, testing and handover around it. No new components, no new interfaces to maintain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>What we need before it starts</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Three things, all before 28 September: the endpoint details in section 3, the firewall and allow-list changes raised, and agreement from ONS to receive from a new sending endpoint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>What good looks like</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Both legs running as configuration rows on one generic engine, zero bespoke components, and Service Operations signing the handover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Why it matters beyond this feed</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>If two similar transfers can both be delivered as configuration, onboarding the rest of the estate is configuration work rather than development work. That is the assumption the wider business case rests on, and it has not been tested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>What could stop it</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Firewall lead time and the ONS agreement. Neither compresses by working harder. If ONS is not ready in time, leg A still delivers inside the window and leg B follows within days of the external path opening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>On the Data Lake migration</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Build now against the current ADR endpoints and re-point to the Data Lake as a configuration change when the warehouse migrates. Option 1 in section 5. Waiting hands our start date to another programme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Decision requested</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Approve the window, name owners on the three critical dependencies, and agree option 1.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:B14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -676,172 +843,172 @@
           <t>Leg B, target, ONS</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Returned by</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Host and port</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="10" t="inlineStr"/>
-      <c r="D5" s="10" t="inlineStr"/>
-      <c r="E5" s="10" t="inlineStr"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
+      <c r="B5" s="9" t="inlineStr"/>
+      <c r="C5" s="9" t="inlineStr"/>
+      <c r="D5" s="9" t="inlineStr"/>
+      <c r="E5" s="9" t="inlineStr"/>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Protocol, SFTP, FTPS, S3 or share</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="10" t="inlineStr"/>
-      <c r="D6" s="10" t="inlineStr"/>
-      <c r="E6" s="10" t="inlineStr"/>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
+      <c r="B6" s="9" t="inlineStr"/>
+      <c r="C6" s="9" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Directory path</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="10" t="inlineStr"/>
-      <c r="D7" s="10" t="inlineStr"/>
-      <c r="E7" s="10" t="inlineStr"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
+      <c r="B7" s="9" t="inlineStr"/>
+      <c r="C7" s="9" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr"/>
+      <c r="E7" s="9" t="inlineStr"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>File name or mask</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="10" t="inlineStr"/>
-      <c r="D8" s="10" t="inlineStr"/>
-      <c r="E8" s="10" t="inlineStr"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="B8" s="9" t="inlineStr"/>
+      <c r="C8" s="9" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Credential type and who issues it</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="10" t="inlineStr"/>
-      <c r="D9" s="10" t="inlineStr"/>
-      <c r="E9" s="10" t="inlineStr"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
+      <c r="B9" s="9" t="inlineStr"/>
+      <c r="C9" s="9" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr"/>
+      <c r="E9" s="9" t="inlineStr"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Host key or certificate</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="10" t="inlineStr"/>
-      <c r="D10" s="10" t="inlineStr"/>
-      <c r="E10" s="10" t="inlineStr"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="B10" s="9" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr"/>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Firewall change needed, which direction</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="10" t="inlineStr"/>
-      <c r="D11" s="10" t="inlineStr"/>
-      <c r="E11" s="10" t="inlineStr"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="B11" s="9" t="inlineStr"/>
+      <c r="C11" s="9" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr"/>
+      <c r="E11" s="9" t="inlineStr"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Source IP the far side must allow</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="10" t="inlineStr"/>
-      <c r="D12" s="10" t="inlineStr"/>
-      <c r="E12" s="10" t="inlineStr"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="B12" s="9" t="inlineStr"/>
+      <c r="C12" s="9" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr"/>
+      <c r="E12" s="9" t="inlineStr"/>
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Archive path</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="10" t="inlineStr"/>
-      <c r="D13" s="10" t="inlineStr"/>
-      <c r="E13" s="10" t="inlineStr"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="B13" s="9" t="inlineStr"/>
+      <c r="C13" s="9" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr"/>
+      <c r="E13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="9" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Quarantine path</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="10" t="inlineStr"/>
-      <c r="D14" s="10" t="inlineStr"/>
-      <c r="E14" s="10" t="inlineStr"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="B14" s="9" t="inlineStr"/>
+      <c r="C14" s="9" t="inlineStr"/>
+      <c r="D14" s="9" t="inlineStr"/>
+      <c r="E14" s="9" t="inlineStr"/>
+      <c r="F14" s="9" t="n"/>
+      <c r="G14" s="9" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Acknowledgement expected</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="10" t="inlineStr"/>
-      <c r="D15" s="10" t="inlineStr"/>
-      <c r="E15" s="10" t="inlineStr"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="B15" s="9" t="inlineStr"/>
+      <c r="C15" s="9" t="inlineStr"/>
+      <c r="D15" s="9" t="inlineStr"/>
+      <c r="E15" s="9" t="inlineStr"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Named contact</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr"/>
-      <c r="C16" s="10" t="inlineStr"/>
-      <c r="D16" s="10" t="inlineStr"/>
-      <c r="E16" s="10" t="inlineStr"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="B16" s="9" t="inlineStr"/>
+      <c r="C16" s="9" t="inlineStr"/>
+      <c r="D16" s="9" t="inlineStr"/>
+      <c r="E16" s="9" t="inlineStr"/>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="9" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:G16"/>
@@ -849,7 +1016,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -896,156 +1063,156 @@
           <t>Done when</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="H3" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>1. Discovery</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Day 1 to 2, 28 to 29 Sep</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Capture the endpoint details in section 3 for both legs. Nothing else. No process mapping, no workshops.</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Every cell in the endpoint table is filled</t>
         </is>
       </c>
-      <c r="E4" s="10" t="n"/>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="10" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>2. Connectivity</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Day 1 to 4, 28 Sep to 1 Oct</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Runs in parallel from day one. Firewall and allow-list changes, credentials, host keys, and a reachability test in both directions.</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>A test file moves end to end on both paths, manually</t>
         </is>
       </c>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>3. Configuration</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Day 5 to 6, 2 and 5 Oct</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Build MFT-INT-001 and MFT-EXT-001 as configuration rows on the generic engine. Schedule, file mask, archive, quarantine, alerts.</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Both rows built, engine gap log empty</t>
         </is>
       </c>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="10" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>4. Testing</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Day 7 to 8, 6 and 7 Oct</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Happy path, file absent, late arrival, duplicate, oversized, scan failure, destination unavailable, credential rejection. Reconcile against the incumbent.</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>All cases evidenced, output byte identical</t>
         </is>
       </c>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
-      <c r="H7" s="10" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>5. Readiness</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Day 9 to 10, 8 and 9 Oct</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Runbook, alerts and escalation. Walk Service Operations through one live failure and recovery. Prove and time the rollback.</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Operations sign the handover, go or no-go issued</t>
         </is>
       </c>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:H8"/>
@@ -1058,7 +1225,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1112,260 +1279,260 @@
           <t>Why it matters</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Owner name</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Raised on</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Endpoint details, all four columns in section 3</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Feed and system owners</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Before day 1</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Discovery is two days only because this arrives complete. If it does not, day 1 becomes chasing, and the window slips</t>
         </is>
       </c>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Firewall and allow-list changes, both legs</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Network security</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Raise now</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>The one item that cannot be compressed by working harder. Standard lead time is longer than the build itself, so it must be raised before the window opens</t>
         </is>
       </c>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="10" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>ONS agreement to receive from a new sending endpoint</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Cross-department liaison</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Raise now</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Leg B cannot be proven without it. If it is not in place, leg A still delivers inside the window and leg B follows</t>
         </is>
       </c>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
-      <c r="H7" s="10" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>ADR to Data Lake migration, agree option 1</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Data Lake programme</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Before day 5</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>See section 5. Option 1 lets the build start on time and treats the re-point as a configuration change</t>
         </is>
       </c>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Credentials and host keys</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Security architecture</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Needed for the connectivity test, not for the build</t>
         </is>
       </c>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="10" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Runtime placement approval</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Platform engineering</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Where the MFT runtime sits for each leg</t>
         </is>
       </c>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Representative or synthetic test file</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Feed owner, ADR</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Day 6</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Testing needs a file with production structure, not production data</t>
         </is>
       </c>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
-      <c r="H11" s="10" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Service Operations availability, half a day</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Service Operations</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Day 9</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>The handover walkthrough is what turns a demo into an accepted service</t>
         </is>
       </c>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="10" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Incumbent path stays live throughout</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Incumbent service owner</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>The MVP runs alongside, it does not cut over</t>
         </is>
       </c>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
-      <c r="H13" s="10" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:H13"/>
@@ -1378,7 +1545,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1425,141 +1592,141 @@
           <t>Option 2</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Decided by</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>What we do</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Migrate the integration now. Move the transfer off legacy IAF onto Boomi, pointing at the existing ADR database and file areas. Re-point to the Data Lake as a configuration change when the warehouse migrates.</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Wait for the warehouse migration to complete, then build once directly against the Data Lake endpoints.</t>
         </is>
       </c>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Start date</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>28 September. Nothing is gated on the Data Lake programme.</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Whenever the warehouse migration lands. Not ours to set.</t>
         </is>
       </c>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="10" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Build effort</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Two days now, plus a one-row endpoint change later.</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Two days, once.</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>What it proves</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Both the transfer and the claim that re-pointing an interface is a configuration change rather than a rebuild.</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>The transfer only.</t>
         </is>
       </c>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>What it costs</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>One config change at migration time, and a short period where the flow points at an endpoint with a known end date.</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>The legacy IAF transfer keeps running on the old platform for the whole duration of the warehouse migration, and the MVP evidence arrives too late to inform the wider onboarding plan.</t>
         </is>
       </c>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Main risk</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>The Data Lake endpoint differs enough that the re-point is not a one-row change. If so, that is a finding worth having early rather than late.</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>The migration slips and the MVP slips with it.</t>
         </is>
       </c>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:F10"/>
@@ -1567,7 +1734,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1607,101 +1774,101 @@
           <t>Needed by</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Owner name</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>Answer</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Confirm the NPS landing area and MWS output area are in migration scope, and the indicative move date</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Data Lake programme</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Day 5</t>
         </is>
       </c>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
-      <c r="F4" s="10" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="9" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Record the Data Lake target endpoints in the configuration row as a known future change, so the re-point is planned rather than discovered</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Integration architecture</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Day 6</t>
         </is>
       </c>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Confirm whether the Maestro chain survives the migration or is replaced by Data Lake ingestion. If replaced, leg A's handover point moves</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Data Lake programme</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Day 5</t>
         </is>
       </c>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="10" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Measure and record the re-point when it happens, as evidence for or against the one-row claim</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Integration architecture</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>At migration</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:F7"/>
@@ -1714,7 +1881,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1749,186 +1916,186 @@
           <t>Met when</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Evidence reference</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>Assessed by</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>SC-1</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Leg A delivers into the ADR landing area, byte identical, three consecutive runs</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n"/>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
-      <c r="F4" s="10" t="n"/>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="9" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>SC-2</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Leg B delivers to ONS, acknowledged, three consecutive runs</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>SC-3</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Both legs are configuration rows on one engine, zero bespoke components</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n"/>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="10" t="n"/>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>SC-4</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>The existing Maestro chain runs unchanged after Boomi delivers</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>SC-5</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>The Insecure IF server hop is absent from the leg B path</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>SC-6</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Non-arrival, transfer failure and scan failure each raise an alert to a named queue, evidenced in test</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>SC-7</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>One audit record per transfer: source, destination, size, checksum, timestamps, outcome</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>SC-8</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Service Operations signs the handover after a live failure and recovery walkthrough</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>SC-9</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Rollback to the incumbent path executed and timed at least once</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>SC-10</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Build effort recorded in hours, separated from time spent waiting on dependencies</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:F13"/>
@@ -1941,7 +2108,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1975,96 +2142,96 @@
           <t>What we do about it</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Firewall change is not complete by day 4</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Raise it now, before the window opens. If it lands late, connectivity slides and everything after it slides with it. This is the single most likely cause of a miss</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n"/>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>ONS endpoint is not agreed in time</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Split the result. Deliver leg A inside the window and report it. Leg B follows within days of the external path opening, because the build is already done</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Endpoint details arrive incomplete</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Day 1 and 2 become chasing. Send the section 3 table out now and treat a complete return as the trigger to open the window</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n"/>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Data Lake migration answers are unclear at day 5</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Proceed on option 1. Build to the current endpoints and record the re-point as a planned one-row change. Do not pause the build waiting for the migration plan</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>No production-like test environment</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Test on the real path with a synthetic file. Say so plainly in the evidence rather than claiming coverage we do not have</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:E8"/>

</xml_diff>

<commit_message>
Rewrite section 0 as a narrative executive summary with at-a-glance, outcomes and three dated decisions
</commit_message>
<xml_diff>
--- a/assets/mft-mvp-tracker.xlsx
+++ b/assets/mft-mvp-tracker.xlsx
@@ -8,24 +8,26 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive view" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endpoint details" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake options" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake conditions" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success criteria" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="At a glance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endpoint details" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake options" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake conditions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success criteria" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Executive view'!$A$4:$B$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Endpoint details'!$A$4:$G$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Plan'!$A$3:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Dependencies'!$A$4:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Data Lake options'!$A$4:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Data Lake conditions'!$A$3:$F$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Success criteria'!$A$3:$F$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Risks'!$A$3:$E$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'At a glance'!$A$4:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Decisions'!$A$4:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Endpoint details'!$A$4:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Plan'!$A$3:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Dependencies'!$A$4:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Data Lake options'!$A$4:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Data Lake conditions'!$A$3:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Success criteria'!$A$3:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Risks'!$A$3:$E$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -620,13 +622,149 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>What could move the date</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>What we do about it</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Firewall change is not complete by day 4</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Raise it now, before the window opens. If it lands late, connectivity slides and everything after it slides with it. This is the single most likely cause of a miss</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>ONS endpoint is not agreed in time</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Split the result. Deliver leg A inside the window and report it. Leg B follows within days of the external path opening, because the build is already done</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Endpoint details arrive incomplete</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Day 1 and 2 become chasing. Send the section 3 table out now and treat a complete return as the trigger to open the window</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Data Lake migration answers are unclear at day 5</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Proceed on option 1. Build to the current endpoints and record the re-point as a planned one-row change. Do not pause the build waiting for the migration plan</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>No production-like test environment</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Test on the real path with a synthetic file. Say so plainly in the evidence rather than claiming coverage we do not have</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:E8"/>
+  <dataValidations count="1">
+    <dataValidation sqref="D4:D8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Open,Mitigating,Closed,Realised"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -636,156 +774,254 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Executive view</t>
+          <t>At a glance</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>The whole argument on one screen. Detail sits in the tabs to the right.</t>
+          <t>The executive summary in the plan document carries the argument. This tab is the reference card behind it.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Question</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Answer</t>
+          <t>Detail</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>What we are doing</t>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Moving one live feed off its legacy transfer mechanisms onto Boomi MFT, and evidencing the result well enough for a go or no-go decision.</t>
+          <t>ADR.040 Migrant Workers Scan. Quarterly, one file per cycle, live in production today</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>On what</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Feed ADR.040, the quarterly Migrant Workers Scan. It is the only feed identified that carries both patterns in a single business flow: NPS to ADR internal, and ADR to ONS external.</t>
+          <t>Two legs. NPS to the ADR landing area, internal. ADR output area to ONS, external</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>When</t>
+          <t>Window</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Monday 28 September to Friday 9 October 2026. Configuration is two days of that.</t>
+          <t>Monday 28 September to Friday 9 October 2026, ten working days</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>What it costs</t>
+          <t>Build effort</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Two days of build effort plus about a week of discovery, testing and handover around it. No new components, no new interfaces to maintain.</t>
+          <t>Two days. Everything else is discovery, testing and handover</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>What we need before it starts</t>
+          <t>New components</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Three things, all before 28 September: the endpoint details in section 3, the firewall and allow-list changes raised, and agreement from ONS to receive from a new sending endpoint.</t>
+          <t>None. Two configuration rows on the existing generic engine</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>What good looks like</t>
+          <t>Side benefit</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Both legs running as configuration rows on one generic engine, zero bespoke components, and Service Operations signing the handover.</t>
+          <t>Removes the Insecure IF server hop from the outbound path, regardless of the platform decision</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Why it matters beyond this feed</t>
+          <t>Known dependency</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>If two similar transfers can both be delivered as configuration, onboarding the rest of the estate is configuration work rather than development work. That is the assumption the wider business case rests on, and it has not been tested.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>What could stop it</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Firewall lead time and the ONS agreement. Neither compresses by working harder. If ONS is not ready in time, leg A still delivers inside the window and leg B follows within days of the external path opening.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>On the Data Lake migration</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Build now against the current ADR endpoints and re-point to the Data Lake as a configuration change when the warehouse migrates. Option 1 in section 5. Waiting hands our start date to another programme.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>Decision requested</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Approve the window, name owners on the three critical dependencies, and agree option 1.</t>
+          <t>ADR to Data Lake migration. Build now, re-point later. Option 1 in section 5</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:B14"/>
+  <autoFilter ref="A4:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>The decisions being asked for</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Three decisions, all before the window opens on 28 September. Nothing else in this workbook matters until these have names against them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>By</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Owner name</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Agreed on</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Name owners for the three critical dependencies: endpoint details, firewall and allow-list changes, and the ONS agreement</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Delivery lead</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Tue 15 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Agree option 1 on the Data Lake migration: build now against the current ADR endpoints, re-point as a configuration change when the warehouse migrates</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Design Authority with the Data Lake programme</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Fri 25 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Approve the two-week window opening 28 September</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Design Authority</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Fri 25 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F7"/>
+  <dataValidations count="1">
+    <dataValidation sqref="E5:E7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Open,In progress,Agreed,Rejected"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1016,7 +1252,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1225,7 +1461,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1545,7 +1781,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1734,7 +1970,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1881,7 +2117,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2106,140 +2342,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>What could move the date</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Risk</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>What we do about it</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E3" s="10" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Firewall change is not complete by day 4</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Raise it now, before the window opens. If it lands late, connectivity slides and everything after it slides with it. This is the single most likely cause of a miss</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="9" t="n"/>
-      <c r="E4" s="9" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>ONS endpoint is not agreed in time</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Split the result. Deliver leg A inside the window and report it. Leg B follows within days of the external path opening, because the build is already done</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Endpoint details arrive incomplete</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Day 1 and 2 become chasing. Send the section 3 table out now and treat a complete return as the trigger to open the window</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Data Lake migration answers are unclear at day 5</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Proceed on option 1. Build to the current endpoints and record the re-point as a planned one-row change. Do not pause the build waiting for the migration plan</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>No production-like test environment</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>Test on the real path with a synthetic file. Say so plainly in the evidence rather than claiming coverage we do not have</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:E8"/>
-  <dataValidations count="1">
-    <dataValidation sqref="D4:D8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Open,Mitigating,Closed,Realised"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Executive summary as three tables: summary, outcomes, decisions
</commit_message>
<xml_diff>
--- a/assets/mft-mvp-tracker.xlsx
+++ b/assets/mft-mvp-tracker.xlsx
@@ -8,26 +8,28 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="At a glance" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endpoint details" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake options" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake conditions" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success criteria" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What we will know" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endpoint details" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake options" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Lake conditions" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success criteria" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'At a glance'!$A$4:$B$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Decisions'!$A$4:$F$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Endpoint details'!$A$4:$G$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Plan'!$A$3:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Dependencies'!$A$4:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Data Lake options'!$A$4:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Data Lake conditions'!$A$3:$F$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Success criteria'!$A$3:$F$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Risks'!$A$3:$E$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Executive summary'!$A$4:$B$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'What we will know'!$A$4:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Decisions'!$A$4:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Endpoint details'!$A$4:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Plan'!$A$3:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Dependencies'!$A$4:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Data Lake options'!$A$4:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Data Lake conditions'!$A$3:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Success criteria'!$A$3:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Risks'!$A$3:$E$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -628,6 +630,233 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Success criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Met when</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Evidence reference</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Assessed by</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>SC-1</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Leg A delivers into the ADR landing area, byte identical, three consecutive runs</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="9" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>SC-2</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Leg B delivers to ONS, acknowledged, three consecutive runs</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>SC-3</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Both legs are configuration rows on one engine, zero bespoke components</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>SC-4</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>The existing Maestro chain runs unchanged after Boomi delivers</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>SC-5</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>The Insecure IF server hop is absent from the leg B path</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>SC-6</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Non-arrival, transfer failure and scan failure each raise an alert to a named queue, evidenced in test</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>SC-7</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>One audit record per transfer: source, destination, size, checksum, timestamps, outcome</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>SC-8</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Service Operations signs the handover after a live failure and recovery walkthrough</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>SC-9</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Rollback to the incumbent path executed and timed at least once</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>SC-10</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Build effort recorded in hours, separated from time spent waiting on dependencies</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:F13"/>
+  <dataValidations count="1">
+    <dataValidation sqref="C4:C13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not assessed,Met,Partially met,Not met"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -764,24 +993,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="104" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>At a glance</t>
+          <t>Executive summary</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>The executive summary in the plan document carries the argument. This tab is the reference card behind it.</t>
+          <t>The same table as section 0 of the plan document.</t>
         </is>
       </c>
     </row>
@@ -800,94 +1029,259 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Candidate</t>
+          <t>What we are doing</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>ADR.040 Migrant Workers Scan. Quarterly, one file per cycle, live in production today</t>
+          <t>Move feed ADR.040 off its legacy transfer mechanisms onto Boomi MFT, and evidence the result well enough for a go or no-go decision.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Two legs. NPS to the ADR landing area, internal. ADR output area to ONS, external</t>
+          <t>ADR.040 Migrant Workers Scan. Quarterly, one file per cycle, live in production. The only feed identified that carries both transfer patterns in a single business flow.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Window</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Monday 28 September to Friday 9 October 2026, ten working days</t>
+          <t>Leg A, NPS into the ADR landing area, internal, replacing UTM. Leg B, ADR output area direct to ONS, external, removing an insecure server hop.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Build effort</t>
+          <t>Why now</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Two days. Everything else is discovery, testing and handover</t>
+          <t>The wider onboarding plan assumes that adding an interface to Boomi MFT is configuration work rather than development work. Nothing has tested that. This tests it twice, inside the estate and across a departmental boundary, for two days of build effort.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>New components</t>
+          <t>Window</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>None. Two configuration rows on the existing generic engine</t>
+          <t>Monday 28 September to Friday 9 October 2026. Ten working days.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Side benefit</t>
+          <t>Build effort</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Removes the Insecure IF server hop from the outbound path, regardless of the platform decision</t>
+          <t>Two days. The other eight are discovery, connectivity, testing and handover.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
+          <t>New components</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>None. Two configuration rows on the existing generic engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Side benefit</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Removes the Insecure IF server hop from the outbound path, whatever the platform decision turns out to be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
           <t>Known dependency</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>ADR to Data Lake migration. Build now, re-point later. Option 1 in section 5</t>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>ADR to Data Lake migration. Build now against the current endpoints and re-point as a configuration change when the warehouse migrates. Option 1 in section 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Main risk</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Firewall changes and the ONS agreement to receive from a new sending endpoint. Lead times that do not compress by working harder, and neither has been started.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Fallback</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>If ONS is not ready in time, leg A still delivers inside the window and leg B follows within days of the external path opening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Cost of not doing it</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>The onboarding estimate behind the wider programme stays an assumption, and the insecure hop stays in the outbound path.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:B11"/>
+  <autoFilter ref="A4:B16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="104" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>What we will know on 9 October</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>The outcomes the two weeks buy. If a row here cannot be answered at the end, the MVP has not finished.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Configuration or code</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Whether a file transfer can be onboarded to Boomi MFT without writing code, evidenced twice rather than argued once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>The real cost</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Onboarding effort in hours, separated from time spent waiting on other teams. That split is the number the wider plan needs and does not have.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Controls</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Whether alerting, audit, quarantine, scanning and rollback hold for an OFFICIAL feed crossing a departmental boundary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Supportability</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Whether Service Operations will accept flows of this kind into support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Migration readiness</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Whether re-pointing an interface at a migrated endpoint is a one-row change, which is what the Data Lake migration will ask of every interface it touches.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:B9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1021,7 +1415,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1252,7 +1646,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1461,7 +1855,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1781,7 +2175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1970,7 +2364,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2115,231 +2509,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="92" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Success criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Ref</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Met when</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>Evidence reference</t>
-        </is>
-      </c>
-      <c r="E3" s="10" t="inlineStr">
-        <is>
-          <t>Assessed by</t>
-        </is>
-      </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>SC-1</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Leg A delivers into the ADR landing area, byte identical, three consecutive runs</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="9" t="n"/>
-      <c r="E4" s="9" t="n"/>
-      <c r="F4" s="9" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>SC-2</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Leg B delivers to ONS, acknowledged, three consecutive runs</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>SC-3</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Both legs are configuration rows on one engine, zero bespoke components</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>SC-4</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>The existing Maestro chain runs unchanged after Boomi delivers</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>SC-5</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>The Insecure IF server hop is absent from the leg B path</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>SC-6</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Non-arrival, transfer failure and scan failure each raise an alert to a named queue, evidenced in test</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>SC-7</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>One audit record per transfer: source, destination, size, checksum, timestamps, outcome</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>SC-8</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Service Operations signs the handover after a live failure and recovery walkthrough</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>SC-9</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Rollback to the incumbent path executed and timed at least once</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>SC-10</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Build effort recorded in hours, separated from time spent waiting on dependencies</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:F13"/>
-  <dataValidations count="1">
-    <dataValidation sqref="C4:C13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Not assessed,Met,Partially met,Not met"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>